<commit_message>
Add mobile app modules, insurance dashboards, and admin UX improvements.
Expand adminapp with stock, service, and insurance management plus sidebar/navigation fixes; add admin and rooftopadmin dashboards, menu access, employee tracking, MSEDCL Smart workflow, and related migrations.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/rooftopadmin/sample_files/pump_capacity_excel.xlsx
+++ b/rooftopadmin/sample_files/pump_capacity_excel.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\ps_projects\vtech\admin\sample_files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\laragon\www\vtech\rooftopadmin\sample_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDAD04E4-A594-4A78-9378-4E02B0A340C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7650"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -24,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>id</t>
   </si>
@@ -32,41 +33,50 @@
     <t>Name</t>
   </si>
   <si>
-    <t>1HP</t>
-  </si>
-  <si>
-    <t>2 HP</t>
-  </si>
-  <si>
-    <t>3 HP</t>
-  </si>
-  <si>
-    <t>5 HP</t>
-  </si>
-  <si>
-    <t>7.5 HP</t>
-  </si>
-  <si>
-    <t>10 HP</t>
+    <t>3.24 kW</t>
+  </si>
+  <si>
+    <t>3.27 kW</t>
+  </si>
+  <si>
+    <t>4.2 kW</t>
+  </si>
+  <si>
+    <t>5.4 kW</t>
+  </si>
+  <si>
+    <t>19.5 kW</t>
+  </si>
+  <si>
+    <t>6 kW</t>
+  </si>
+  <si>
+    <t>4.9 kW</t>
+  </si>
+  <si>
+    <t>3.3 kW</t>
+  </si>
+  <si>
+    <t>4.4 kW</t>
+  </si>
+  <si>
+    <t>2.2 kW</t>
+  </si>
+  <si>
+    <t>5.5 kW</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -89,9 +99,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -371,11 +380,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:B12"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -383,52 +392,92 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>16</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>17</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>18</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5">
-        <v>19</v>
-      </c>
-      <c r="B5" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="B5" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6">
-        <v>20</v>
-      </c>
-      <c r="B6" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="B6" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7">
-        <v>21</v>
-      </c>
-      <c r="B7" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="B7" t="s">
         <v>7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A8">
+        <v>125</v>
+      </c>
+      <c r="B8" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A9">
+        <v>126</v>
+      </c>
+      <c r="B9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A10">
+        <v>127</v>
+      </c>
+      <c r="B10" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A11">
+        <v>128</v>
+      </c>
+      <c r="B11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A12">
+        <v>129</v>
+      </c>
+      <c r="B12" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>